<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-08 Le ruban rouge
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-08.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-08.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le ruban dans le rayon</t>
+          <t>Le ruban rouge</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, radio et rayon de poussière</t>
+          <t>salon, radio sur la commode, chanson, ruban rouge, linge près de la fenêtre, clic du bois</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut dessiner un grand rond lent avec le ruban rouge dans le rayon de soleil. Sarah arrive avec beaucoup d'énergie. Le ruban s'enroule à la chaise. Ils jouent, ils attendent, Aniss demande à maman. Le rond est lent, et il est là.</t>
+          <t>Le bois de la commode fait clic sous la radio. Sur le bois, un éclat de commode brille. Aniss veut un grand rond lent, maintenant, pendant la chanson. Sarah saute trop, le ruban s'enroule au pied. Sourire parti, poitrine, papa accroupi. Aniss refuse de foncer, attend, demande. Merci vécu. Ruban trop vite vers la radio. Un éclat de commode tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La radio craque, puis trouve une chanson. Le bouton est lisse sous le doigt de papa. Tu entends la chanson, Aniss ? Oui. Elle est douce. Un ruban rouge glisse de la chaise. Il tombe comme une petite rivière. Le tapis est épais et beige. Maman ouvre un peu la fenêtre. L'air sent le linge sec. Un rayon traverse le salon. Il est plein de poussière brillante. En ce moment, Aniss prend le ruban. Il est long. Il sent un peu le bois de la chaise. Je veux danser. Un grand rond, lent. On danse avec le ruban, alors. Aniss lève le bras. Le ruban dessine un tout petit arc. Sarah arrive. Elle saute sur place. Elle a beaucoup d'énergie. Les pieds tapent le tapis. Elle saute, papa. C'est son énergie. Ce n'est pas une faute. Aniss tend le ruban. Ils dansent. Sarah tourne vite. Le ruban s'enroule autour de la chaise. Oh. Le rond. Sarah rebondit encore. Aniss regarde maman.</t>
+          <t>Le bois de la commode fait clic, sous la radio. Ça craque une fois, sec et chaud. J'ai entendu le clic. Près de la radio, Aniss ? Oui, papa. Papa tourne le bouton, lisse sous le doigt. Une chanson arrive, un peu voilée. Elle est douce. Tu l'entends, la chanson ? Oui. On danse un peu, alors. Maman plie un linge près de la fenêtre. L'air sent le linge sec. Ça sent le savon, maman. Tu le sens, Aniss ? Un peu, maman. Sur le bois, un éclat de commode brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un ruban rouge dort contre la radio. Le tissu est long, un peu tiède. Il est chaud, papa. Le bois est dessous ? Oui. En ce moment, Aniss prend le ruban. Je veux danser, maintenant ! Un grand rond, lent, pendant la chanson. Un petit rond, là ? Un grand rond. La radio reste sur la commode. Après le rond. Aniss lève le bras. Le ruban dessine un arc, bas. Sarah arrive dans le salon. Elle court un peu, pieds légers. Je saute ! Sarah saute trop, trop près du ruban. Tu danses avec moi ? Oui. Sarah tourne trop vite. Le ruban s'enroule au pied de la commode. La radio penche, un peu. Oh. Le rond. Il est tombé. Aniss tient le ruban contre lui. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Sarah, Aniss ? Oui, papa. Tes mains tiennent le ruban, Aniss ? Un peu, maman. L'éclat de commode tremble, puis tient. Sarah tape des pieds près de la commode. Elle saute partout, papa. Aniss regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La radio craque, puis trouve une chanson. Le bouton est lisse sous le doigt de papa. Tu entends la chanson, Aniss ? Oui. Elle est douce. Un ruban rouge glisse de la chaise. Il tombe comme une petite rivière. Le tapis est épais et beige. Maman ouvre un peu la fenêtre. L'air sent le linge sec. Un rayon traverse le salon. Il est plein de poussière brillante. En ce moment, Aniss prend le ruban. Il est long. Il sent un peu le bois de la chaise. Je veux danser. Un grand rond, lent. On danse avec le ruban, alors. Aniss lève le bras. Le ruban dessine un tout petit arc. Sarah arrive. Elle saute sur place. Elle a beaucoup d'énergie. Les pieds tapent le tapis. Elle saute, papa. C'est son énergie. Ce n'est pas une faute. Aniss tend le ruban. Ils dansent. Sarah tourne vite. Le ruban s'enroule autour de la chaise. Oh. Le rond. Sarah rebondit encore. Aniss regarde maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le bois de la commode fait clic, sous la radio. Ça craque une fois, sec et chaud. J'ai entendu le clic. Près de la radio, Aniss ? Oui, papa. Papa tourne le bouton, lisse sous le doigt. Une chanson arrive, un peu voilée. Elle est douce. Tu l'entends, la chanson ? Oui. On danse un peu, alors. Maman plie un linge près de la fenêtre. L'air sent le linge sec. Ça sent le savon, maman. Tu le sens, Aniss ? Un peu, maman. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de commode&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un ruban rouge dort contre la radio. Le tissu est long, un peu tiède. Il est chaud, papa. Le bois est dessous ? Oui. En ce moment, Aniss prend le ruban. Je veux danser, maintenant ! Un grand rond, lent, pendant la chanson. Un petit rond, là ? Un grand rond. La radio reste sur la commode. Après le rond. Aniss lève le bras. Le ruban dessine un arc, bas. Sarah arrive dans le salon. Elle court un peu, pieds légers. Je saute ! Sarah saute trop, trop près du ruban. Tu danses avec moi ? Oui. Sarah tourne trop vite. Le ruban s'enroule au pied de la commode. La radio penche, un peu. Oh. Le rond. Il est tombé. Aniss tient le ruban contre lui. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Sarah, Aniss ? Oui, papa. Tes mains tiennent le ruban, Aniss ? Un peu, maman. L'éclat de commode tremble, puis tient. Sarah tape des pieds près de la commode. Elle saute partout, papa. Aniss regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maman met une chanson dans le salon. Bruno tient un ruban. Noé arrive. Il saute sur place. Il a beaucoup d'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Les pieds tapent le tapis. Bruno le regarde. Maman dit : beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. Bruno tend un ruban. Ils dansent. Noé tourne vite. Bruno dit : on peut attendre. Noé souffle. Il attend son tour pour le grand ruban. Ils jouent. Plus tard, Noé rebondit encore. Ce n'est pas une faute. Bruno va vers maman. Il demande à un adulte. Maman propose les coussins. On peut jouer ou attendre. Bruno dit : Noé a de l'énergie. Maman dit : ce n'est pas une faute. Ils s'assoient un moment. Puis ils reprennent le ruban. [pause]</t>
+          <t>Le bois de la commode fait clic, sous la radio. Ça craque une fois, sec et chaud. J'ai entendu le clic. Près de la radio, Aniss ? Oui, papa. Papa tourne le bouton, lisse sous le doigt. Une chanson arrive, un peu voilée. Elle est douce. Tu l'entends, la chanson ? Oui. On danse un peu, alors. Maman plie un linge près de la fenêtre. L'air sent le linge sec. Ça sent le savon, maman. Tu le sens, Aniss ? Un peu, maman. Sur le bois, un &lt;emphasis&gt;éclat de commode&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Un ruban rouge dort contre la radio. Le tissu est long, un peu tiède. Il est chaud, papa. Le bois est dessous ? Oui. En ce moment, Aniss prend le ruban. Je veux danser, maintenant ! Un grand rond, lent, pendant la chanson. Un petit rond, là ? Un grand rond. La radio reste sur la commode. Après le rond. Aniss lève le bras. Le ruban dessine un arc, bas. Sarah arrive dans le salon. Elle court un peu, pieds légers. Je saute ! Sarah saute trop, trop près du ruban. Tu danses avec moi ? Oui. Sarah tourne trop vite. Le ruban s'enroule au pied de la commode. La radio penche, un peu. Oh. Le rond. Il est tombé. Aniss tient le ruban contre lui. Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Sarah, Aniss ? Oui, papa. Tes mains tiennent le ruban, Aniss ? Un peu, maman. L'éclat de commode tremble, puis tient. Sarah tape des pieds près de la commode. Elle saute partout, papa. Aniss regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de commode</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,44 +1321,77 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_un_grand_rond_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La radio craque, puis trouve une chanson.
-narrateur|Le bouton est lisse sous le doigt de papa.
-papa|Tu entends la chanson, Aniss ?
+          <t>narrateur|Le bois de la commode fait clic, sous la radio.
+narrateur|Ça craque une fois, sec et chaud.
+enfant-m|J'ai entendu le clic.
+papa|Près de la radio, Aniss ?
+enfant-m|Oui, papa.
+narrateur|Papa tourne le bouton, lisse sous le doigt.
+narrateur|Une chanson arrive, un peu voilée.
+enfant-m|Elle est douce.
+papa|Tu l'entends, la chanson ?
 enfant-m|Oui.
-enfant-m|Elle est douce.
-narrateur|Un ruban rouge glisse de la chaise.
-narrateur|Il tombe comme une petite rivière.
-narrateur|Le tapis est épais et beige.
-narrateur|Maman ouvre un peu la fenêtre.
-maman|L'air sent le linge sec.
-narrateur|Un rayon traverse le salon.
-narrateur|Il est plein de poussière brillante.
+maman|On danse un peu, alors.
+narrateur|Maman plie un linge près de la fenêtre.
+narrateur|L'air sent le linge sec.
+enfant-m|Ça sent le savon, maman.
+maman|Tu le sens, Aniss ?
+enfant-m|Un peu, maman.
+narrateur|Sur le bois, un éclat de commode brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Un ruban rouge dort contre la radio.
+narrateur|Le tissu est long, un peu tiède.
+enfant-m|Il est chaud, papa.
+papa|Le bois est dessous ?
+enfant-m|Oui.
 narrateur|En ce moment, Aniss prend le ruban.
-narrateur|Il est long.
-narrateur|Il sent un peu le bois de la chaise.
-enfant-m|Je veux danser.
-enfant-m|Un grand rond, lent.
-maman|On danse avec le ruban, alors.
+enfant-m|Je veux danser, maintenant !
+enfant-m|Un grand rond, lent, pendant la chanson.
+papa|Un petit rond, là ?
+enfant-m|Un grand rond.
+maman|La radio reste sur la commode.
+enfant-m|Après le rond.
 narrateur|Aniss lève le bras.
-narrateur|Le ruban dessine un tout petit arc.
-narrateur|Sarah arrive.
-narrateur|Elle saute sur place.
-narrateur|Elle a beaucoup d'énergie.
-narrateur|Les pieds tapent le tapis.
-enfant-m|Elle saute, papa.
-papa|C'est son énergie.
-papa|Ce n'est pas une faute.
-narrateur|Aniss tend le ruban.
-narrateur|Ils dansent.
-narrateur|Sarah tourne vite.
-narrateur|Le ruban s'enroule autour de la chaise.
+narrateur|Le ruban dessine un arc, bas.
+narrateur|Sarah arrive dans le salon.
+narrateur|Elle court un peu, pieds légers.
+enfant-f|Je saute !
+narrateur|Sarah saute trop, trop près du ruban.
+enfant-m|Tu danses avec moi ?
+enfant-f|Oui.
+narrateur|Sarah tourne trop vite.
+narrateur|Le ruban s'enroule au pied de la commode.
+narrateur|La radio penche, un peu.
 enfant-m|Oh.
 enfant-m|Le rond.
-narrateur|Sarah rebondit encore.
-narrateur|Aniss regarde maman.</t>
+enfant-f|Il est tombé.
+narrateur|Aniss tient le ruban contre lui.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Sarah, Aniss ?
+enfant-m|Oui, papa.
+maman|Tes mains tiennent le ruban, Aniss ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de commode tremble, puis tient.
+narrateur|Sarah tape des pieds près de la commode.
+enfant-m|Elle saute partout, papa.
+narrateur|Aniss regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>radio,commode</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1423,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah a de l'énergie. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Noé a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1458,18 +1491,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,11 +1517,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1499,23 +1532,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1524,23 +1557,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=sarah_a_de_l_energie; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss va vers maman. Maman, on fait quoi ? On danse avec le ruban. On attend le grand tour. Tu es venu me voir. On prend les coussins. Ils s'assoient un moment. Le tapis étouffe les pas. L'énergie est encore là. Ce n'est pas une faute. On peut attendre. Sarah souffle. Elle attend son tour pour le grand ruban. C'est à Aniss. Aniss défait le ruban de la chaise. Il est doux entre les doigts. Puis ils reprennent le ruban. La chanson est plus douce. Le ruban fait un grand rond ? Un grand rond. Aniss fait un rond lent. Le ruban passe dans le rayon. Il devient tout lumineux. Sarah tend le ruban. J'attends. Elle attend. Puis elle fait un rond, plus lent. Ils jouent. Le rayon traverse le ruban. Il est tout rouge. Et tout lumineux. Encore un rond, plus calme ? Plus calme.</t>
+          <t>Aniss veut le grand rond, tout de suite. Je le refais, maintenant ! Il avance trop vite vers Sarah. Les mots se bousculent dans sa bouche. Attends. Sarah tape des pieds, trop près. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le ruban, un instant. Il écoute la chanson de la radio. Tu veux le rond avec Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On passe le ruban, puis on tourne. D'accord. Aniss tend le ruban, sans se presser. Il reste un moment, les mains ouvertes. Sarah souffle. Le mien. Sarah prend le ruban, plus lentement. Merci, Aniss. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le ruban se défait du pied de la commode. Le rond. Il fait un cercle, là ? Oui, là. Aniss lève le bras, sans se presser. Le tissu est doux, contre la peau. Tes mains sont au chaud, Aniss ? Un peu, maman. Sarah s'assoit, puis se relève. J'y vais. On tourne près de la radio ? La radio reste sur le bois. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss va vers maman. Maman, on fait quoi ? On danse avec le ruban. On attend le grand tour. Tu es venu me voir. On prend les coussins. Ils s'assoient un moment. Le tapis étouffe les pas. L'énergie est encore là. Ce n'est pas une faute. On peut attendre. Sarah souffle. Elle attend son tour pour le grand ruban. C'est à Aniss. Aniss défait le ruban de la chaise. Il est doux entre les doigts. Puis ils reprennent le ruban. La chanson est plus douce. Le ruban fait un grand rond ? Un grand rond. Aniss fait un rond lent. Le ruban passe dans le rayon. Il devient tout lumineux. Sarah tend le ruban. J'attends. Elle attend. Puis elle fait un rond, plus lent. Ils jouent. Le rayon traverse le ruban. Il est tout rouge. Et tout lumineux. Encore un rond, plus calme ? Plus calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut le grand rond, tout de suite. Je le refais, maintenant ! Il avance trop vite vers Sarah. Les mots se bousculent dans sa bouche. Attends. Sarah tape des pieds, trop près. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le &lt;emphasis level="moderate"&gt;ruban&lt;/emphasis&gt;, un instant. Il écoute la chanson de la radio. Tu veux le rond avec Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On passe le ruban, puis on tourne. D'accord. Aniss tend le ruban, sans se presser. Il reste un moment, les mains ouvertes. Sarah souffle. Le mien. Sarah prend le ruban, plus lentement. Merci, Aniss. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le ruban se défait du pied de la commode. Le rond. Il fait un cercle, là ? Oui, là. Aniss lève le bras, sans se presser. Le tissu est doux, contre la peau. Tes mains sont au chaud, Aniss ? Un peu, maman. Sarah s'assoit, puis se relève. J'y vais. On tourne près de la radio ? La radio reste sur le bois. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Noé a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Bruno a joué. Il a su attendre. Il a demandé à un adulte. [pause]</t>
+          <t>Aniss veut le grand rond, tout de suite. Je le refais, maintenant ! Il avance trop vite vers Sarah. Les mots se bousculent dans sa bouche. Attends. Sarah tape des pieds, trop près. Oh. Le sourire ne revient pas. Aniss refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le &lt;emphasis&gt;ruban&lt;/emphasis&gt;, un instant. Il écoute la chanson de la radio. Tu veux le rond avec Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On passe le ruban, puis on tourne. D'accord. Aniss tend le ruban, sans se presser. Il reste un moment, les mains ouvertes. Sarah souffle. Le mien. Sarah prend le ruban, plus lentement. Merci, Aniss. Papa a vu les deux, au salon. Le tissu est tiède, sous les doigts. Il est chaud. Le ruban se défait du pied de la commode. Le rond. Il fait un cercle, là ? Oui, là. Aniss lève le bras, sans se presser. Le tissu est doux, contre la peau. Tes mains sont au chaud, Aniss ? Un peu, maman. Sarah s'assoit, puis se relève. J'y vais. On tourne près de la radio ? La radio reste sur le bois. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1663,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1671,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1664,30 +1697,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>ruban</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1696,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,44 +1745,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_attend_demande; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss va vers maman.
-enfant-m|Maman, on fait quoi ?
-maman|On danse avec le ruban.
-maman|On attend le grand tour.
-maman|Tu es venu me voir.
-maman|On prend les coussins.
-narrateur|Ils s'assoient un moment.
-narrateur|Le tapis étouffe les pas.
-papa|L'énergie est encore là.
-papa|Ce n'est pas une faute.
-enfant-m|On peut attendre.
+          <t>narrateur|Aniss veut le grand rond, tout de suite.
+enfant-m|Je le refais, maintenant !
+narrateur|Il avance trop vite vers Sarah.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Attends.
+narrateur|Sarah tape des pieds, trop près.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Aniss refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le ruban, un instant.
+narrateur|Il écoute la chanson de la radio.
+papa|Tu veux le rond avec Sarah ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Papa, on fait quoi ?
+papa|On passe le ruban, puis on tourne.
+enfant-m|D'accord.
+narrateur|Aniss tend le ruban, sans se presser.
+narrateur|Il reste un moment, les mains ouvertes.
 narrateur|Sarah souffle.
-narrateur|Elle attend son tour pour le grand ruban.
-maman|C'est à Aniss.
-narrateur|Aniss défait le ruban de la chaise.
-narrateur|Il est doux entre les doigts.
-narrateur|Puis ils reprennent le ruban.
-narrateur|La chanson est plus douce.
-papa|Le ruban fait un grand rond ?
-enfant-m|Un grand rond.
-narrateur|Aniss fait un rond lent.
-narrateur|Le ruban passe dans le rayon.
-narrateur|Il devient tout lumineux.
-narrateur|Sarah tend le ruban.
-enfant-f|J'attends.
-narrateur|Elle attend.
-narrateur|Puis elle fait un rond, plus lent.
-narrateur|Ils jouent.
-narrateur|Le rayon traverse le ruban.
-enfant-m|Il est tout rouge.
-maman|Et tout lumineux.
-papa|Encore un rond, plus calme ?
-enfant-m|Plus calme.</t>
+enfant-f|Le mien.
+narrateur|Sarah prend le ruban, plus lentement.
+papa|Merci, Aniss.
+narrateur|Papa a vu les deux, au salon.
+maman|Le tissu est tiède, sous les doigts.
+enfant-m|Il est chaud.
+narrateur|Le ruban se défait du pied de la commode.
+enfant-m|Le rond.
+papa|Il fait un cercle, là ?
+enfant-m|Oui, là.
+narrateur|Aniss lève le bras, sans se presser.
+narrateur|Le tissu est doux, contre la peau.
+maman|Tes mains sont au chaud, Aniss ?
+enfant-m|Un peu, maman.
+narrateur|Sarah s'assoit, puis se relève.
+enfant-f|J'y vais.
+enfant-m|On tourne près de la radio ?
+maman|La radio reste sur le bois.
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>ruban</t>
         </is>
       </c>
     </row>
@@ -1776,17 +1821,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On baisse la chanson ? Oui, maman. Maman baisse la chanson. Aniss range un ruban. Le ruban rouge va sur la chaise ? Oui. Le rayon devient tout calme. Le rond était lent. Et lumineux. On l'a vu, tous les deux. Sarah pose le bout du ruban. Il retombe comme une rivière.</t>
+          <t>Ils restent près de la commode. La radio fait clic, sous le bois. À moi ! Sarah tire le ruban trop vite. On se passe le ruban, près du bois ? Oui, maman. Aniss envoie le ruban trop vite. Le ruban penche vers la radio. Ça tombe ! Attends. Aniss avance les mains, trop vite. Puis il s'arrête net. Aniss refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le bois, un instant. Il écoute le clic de la radio. Sur le bois, un éclat de commode luit. Là, sur la commode. Tu prends le ruban, Sarah ? Sarah ne dit rien. Elle tend les mains, sans parler. Oui. Aniss envoie le ruban, sans se presser. Sarah le renvoie, plus lentement. Le ruban est lisse et chaud. Tu le vois, le ruban ? Oui, papa. La radio est sur le bois ? Oui, maman. Ils font un rond, plus lent. Aniss lève le bras. Sarah lève le sien. Le rond tient, Aniss ? Oui, papa. Un filet de chanson passe sur le tissu. Il allume le ruban.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On baisse la chanson ? Oui, maman. Maman baisse la chanson. Aniss range un ruban. Le ruban rouge va sur la chaise ? Oui. Le rayon devient tout calme. Le rond était lent. Et lumineux. On l'a vu, tous les deux. Sarah pose le bout du ruban. Il retombe comme une rivière.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près de la commode. La radio fait clic, sous le bois. À moi ! Sarah tire le ruban trop vite. On se passe le ruban, près du bois ? Oui, maman. Aniss envoie le ruban trop vite. Le ruban penche vers la radio. Ça tombe ! Attends. Aniss avance les mains, trop vite. Puis il s'arrête net. Aniss refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le bois, un instant. Il écoute le clic de la radio. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de commode&lt;/emphasis&gt; luit. Là, sur la commode. Tu prends le ruban, Sarah ? Sarah ne dit rien. Elle tend les mains, sans parler. Oui. Aniss envoie le ruban, sans se presser. Sarah le renvoie, plus lentement. Le ruban est lisse et chaud. Tu le vois, le ruban ? Oui, papa. La radio est sur le bois ? Oui, maman. Ils font un rond, plus lent. Aniss lève le bras. Sarah lève le sien. Le rond tient, Aniss ? Oui, papa. Un filet de chanson passe sur le tissu. Il allume le ruban.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman baisse la chanson. Bruno range un ruban. [pause]</t>
+          <t>Ils restent près de la commode. La radio fait clic, sous le bois. À moi ! Sarah tire le ruban trop vite. On se passe le ruban, près du bois ? Oui, maman. Aniss envoie le ruban trop vite. Le ruban penche vers la radio. Ça tombe ! Attends. Aniss avance les mains, trop vite. Puis il s'arrête net. Aniss refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le bois, un instant. Il écoute le clic de la radio. Sur le bois, un &lt;emphasis&gt;éclat de commode&lt;/emphasis&gt; luit. Là, sur la commode. Tu prends le ruban, Sarah ? Sarah ne dit rien. Elle tend les mains, sans parler. Oui. Aniss envoie le ruban, sans se presser. Sarah le renvoie, plus lentement. Le ruban est lisse et chaud. Tu le vois, le ruban ? Oui, papa. La radio est sur le bois ? Oui, maman. Ils font un rond, plus lent. Aniss lève le bras. Sarah lève le sien. Le rond tient, Aniss ? Oui, papa. Un filet de chanson passe sur le tissu. Il allume le ruban. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1833,7 +1878,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1841,10 +1886,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1865,28 +1910,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de commode</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1895,10 +1944,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1909,21 +1958,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=ruban_trop_vite_vers_la_radio; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On baisse la chanson ?
+          <t>narrateur|Ils restent près de la commode.
+narrateur|La radio fait clic, sous le bois.
+enfant-f|À moi !
+narrateur|Sarah tire le ruban trop vite.
+maman|On se passe le ruban, près du bois ?
 enfant-m|Oui, maman.
-narrateur|Maman baisse la chanson.
-narrateur|Aniss range un ruban.
-papa|Le ruban rouge va sur la chaise ?
-enfant-m|Oui.
-narrateur|Le rayon devient tout calme.
-maman|Le rond était lent.
-enfant-m|Et lumineux.
-papa|On l'a vu, tous les deux.
-narrateur|Sarah pose le bout du ruban.
-narrateur|Il retombe comme une rivière.</t>
+narrateur|Aniss envoie le ruban trop vite.
+narrateur|Le ruban penche vers la radio.
+enfant-m|Ça tombe !
+enfant-f|Attends.
+narrateur|Aniss avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Aniss refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le bois, un instant.
+narrateur|Il écoute le clic de la radio.
+narrateur|Sur le bois, un éclat de commode luit.
+enfant-m|Là, sur la commode.
+enfant-m|Tu prends le ruban, Sarah ?
+narrateur|Sarah ne dit rien.
+narrateur|Elle tend les mains, sans parler.
+enfant-f|Oui.
+narrateur|Aniss envoie le ruban, sans se presser.
+narrateur|Sarah le renvoie, plus lentement.
+narrateur|Le ruban est lisse et chaud.
+papa|Tu le vois, le ruban ?
+enfant-m|Oui, papa.
+maman|La radio est sur le bois ?
+enfant-m|Oui, maman.
+narrateur|Ils font un rond, plus lent.
+narrateur|Aniss lève le bras.
+narrateur|Sarah lève le sien.
+papa|Le rond tient, Aniss ?
+enfant-m|Oui, papa.
+maman|Un filet de chanson passe sur le tissu.
+enfant-m|Il allume le ruban.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>radio,ruban</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2033,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le ruban rouge dort sur la chaise. La radio fait un tout petit souffle. Le rond est resté dans le rayon. Un grand rond lent.</t>
+          <t>Ils s'assoient près du bois. La chanson s'arrête, Aniss ? Oui, maman. Tu poses le ruban sur le bois ? Oui, papa. Aniss pose le ruban, près de la radio. Le rouge sent le bois. Tu le sens, le bois ? Oui, maman. Le rond reste un peu, de travers. Il a tenu, pendant la chanson. Le ruban est resté. La radio fait un petit souffle. Le ruban rouge fait de l'ombre. On y retourne, après. Un éclat de commode tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le ruban rouge dort sur la chaise. La radio fait un tout petit souffle. Le rond est resté dans le rayon. Un grand rond lent.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'assoient près du bois. La chanson s'arrête, Aniss ? Oui, maman. Tu poses le ruban sur le bois ? Oui, papa. Aniss pose le ruban, près de la radio. Le rouge sent le bois. Tu le sens, le bois ? Oui, maman. Le rond reste un peu, de travers. Il a tenu, pendant la chanson. Le ruban est resté. La radio fait un petit souffle. Le ruban rouge fait de l'ombre. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de commode&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'assoient près du bois. La chanson s'arrête, Aniss ? Oui, maman. Tu poses le ruban sur le bois ? Oui, papa. Aniss pose le ruban, près de la radio. Le rouge sent le bois. Tu le sens, le bois ? Oui, maman. Le rond reste un peu, de travers. Il a tenu, pendant la chanson. Le ruban est resté. La radio fait un petit souffle. Le ruban rouge fait de l'ombre. On y retourne, après. Un &lt;emphasis&gt;éclat de commode&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,18 +2090,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2110,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2124,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de commode</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2147,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,27 +2160,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le ruban rouge dort sur la chaise.
-narrateur|La radio fait un tout petit souffle.
-papa|Le rond est resté dans le rayon.
-enfant-m|Un grand rond lent.</t>
+          <t>narrateur|Ils s'assoient près du bois.
+maman|La chanson s'arrête, Aniss ?
+enfant-m|Oui, maman.
+papa|Tu poses le ruban sur le bois ?
+enfant-m|Oui, papa.
+narrateur|Aniss pose le ruban, près de la radio.
+enfant-m|Le rouge sent le bois.
+maman|Tu le sens, le bois ?
+enfant-m|Oui, maman.
+papa|Le rond reste un peu, de travers.
+enfant-m|Il a tenu, pendant la chanson.
+enfant-f|Le ruban est resté.
+narrateur|La radio fait un petit souffle.
+narrateur|Le ruban rouge fait de l'ombre.
+enfant-m|On y retourne, après.
+narrateur|Un éclat de commode tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radio</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2199,6 +2307,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>